<commit_message>
Expansion on classification flags as well as improving flagging reach
</commit_message>
<xml_diff>
--- a/FR testing.xlsx
+++ b/FR testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myecf-my.sharepoint.com/personal/oadode_ecf_ca/Documents/Desktop/Discretionary FR Scripting/ECF-Discretionary-FR-Scripting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="11_1AE67D4D96B88102FD7E0298CDC6DCCA3A23EDAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B61506B-A298-4071-98D0-8A5F9D04A873}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_1AE67D4D96B88102FD7E0298CDC6DCCA3A23EDAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BA90E4F-7B1B-4E75-8B7B-EA1BFA7F02FF}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19247,7 +19247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2025</v>
       </c>
@@ -19297,7 +19297,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2025</v>
       </c>
@@ -19485,7 +19485,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2025</v>
       </c>
@@ -19535,7 +19535,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2025</v>
       </c>
@@ -19629,7 +19629,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2025</v>
       </c>
@@ -19972,7 +19972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2025</v>
       </c>
@@ -20113,7 +20113,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="25" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2025</v>
       </c>
@@ -20236,7 +20236,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="28" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2025</v>
       </c>
@@ -20289,7 +20289,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="29" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>2025</v>
       </c>
@@ -20436,7 +20436,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="32" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>2025</v>
       </c>
@@ -20773,7 +20773,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="40" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>2025</v>
       </c>
@@ -21160,7 +21160,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="49" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>2025</v>
       </c>
@@ -21201,7 +21201,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="50" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>2025</v>
       </c>
@@ -21251,7 +21251,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="51" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>2025</v>
       </c>
@@ -21301,7 +21301,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="52" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>2025</v>
       </c>
@@ -21500,7 +21500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>2025</v>
       </c>
@@ -21532,7 +21532,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="58" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>2025</v>
       </c>
@@ -21576,7 +21576,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="59" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>2025</v>
       </c>
@@ -21664,7 +21664,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="61" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>2025</v>
       </c>
@@ -21746,7 +21746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>2025</v>
       </c>
@@ -21825,7 +21825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>2025</v>
       </c>
@@ -21878,7 +21878,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="66" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>2025</v>
       </c>
@@ -21978,7 +21978,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="68" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>2025</v>
       </c>
@@ -22069,7 +22069,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="70" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>2025</v>
       </c>
@@ -22110,7 +22110,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="71" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>2025</v>
       </c>
@@ -22160,7 +22160,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="72" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>2025</v>
       </c>
@@ -22462,7 +22462,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="79" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>2025</v>
       </c>
@@ -22829,7 +22829,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="87" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>2025</v>
       </c>
@@ -23046,7 +23046,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="92" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>2025</v>
       </c>
@@ -23131,7 +23131,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="94" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>2025</v>
       </c>
@@ -23216,7 +23216,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="96" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>2025</v>
       </c>
@@ -23263,7 +23263,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="97" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>2025</v>
       </c>
@@ -23545,7 +23545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>2025</v>
       </c>
@@ -23592,7 +23592,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="104" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>2025</v>
       </c>
@@ -23924,7 +23924,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="111" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>2025</v>
       </c>
@@ -24308,7 +24308,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="120" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>2025</v>
       </c>
@@ -24352,7 +24352,7 @@
         <v>865</v>
       </c>
     </row>
-    <row r="121" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>2025</v>
       </c>
@@ -24724,7 +24724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>2025</v>
       </c>
@@ -24771,7 +24771,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="131" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>2025</v>
       </c>
@@ -24999,7 +24999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>2025</v>
       </c>
@@ -25242,7 +25242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>2025</v>
       </c>
@@ -25921,7 +25921,7 @@
         <v>1078</v>
       </c>
     </row>
-    <row r="160" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>2025</v>
       </c>
@@ -26021,7 +26021,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="162" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>2025</v>
       </c>
@@ -26071,7 +26071,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="163" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>2025</v>
       </c>
@@ -26218,7 +26218,7 @@
         <v>1125</v>
       </c>
     </row>
-    <row r="166" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>2025</v>
       </c>
@@ -27332,7 +27332,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="192" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>2025</v>
       </c>
@@ -27411,7 +27411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>2025</v>
       </c>
@@ -27461,7 +27461,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="195" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>2025</v>
       </c>
@@ -27593,7 +27593,7 @@
         <v>1321</v>
       </c>
     </row>
-    <row r="198" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>2025</v>
       </c>
@@ -27757,7 +27757,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="202" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>2025</v>
       </c>
@@ -27901,7 +27901,7 @@
         <v>1365</v>
       </c>
     </row>
-    <row r="205" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>2025</v>
       </c>
@@ -27951,7 +27951,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="206" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>2025</v>
       </c>
@@ -28001,7 +28001,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="207" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>2025</v>
       </c>
@@ -28086,7 +28086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>2025</v>
       </c>
@@ -28303,7 +28303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>2025</v>
       </c>
@@ -28432,7 +28432,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="217" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>2025</v>
       </c>
@@ -28485,7 +28485,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="218" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>2025</v>
       </c>
@@ -28661,7 +28661,7 @@
         <v>1473</v>
       </c>
     </row>
-    <row r="222" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>2025</v>
       </c>
@@ -28702,7 +28702,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="223" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>2025</v>
       </c>
@@ -28743,7 +28743,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="224" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>2025</v>
       </c>
@@ -28963,7 +28963,7 @@
         <v>1521</v>
       </c>
     </row>
-    <row r="229" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>2025</v>
       </c>
@@ -29060,7 +29060,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="231" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>2025</v>
       </c>
@@ -29160,7 +29160,7 @@
         <v>884</v>
       </c>
     </row>
-    <row r="233" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>2025</v>
       </c>
@@ -29210,7 +29210,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="234" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>2025</v>
       </c>
@@ -29310,7 +29310,7 @@
         <v>1570</v>
       </c>
     </row>
-    <row r="236" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>2025</v>
       </c>
@@ -29515,7 +29515,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="241" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>2025</v>
       </c>
@@ -29725,7 +29725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>2025</v>
       </c>
@@ -30196,7 +30196,7 @@
         <v>1693</v>
       </c>
     </row>
-    <row r="259" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>2025</v>
       </c>
@@ -30290,7 +30290,7 @@
         <v>1705</v>
       </c>
     </row>
-    <row r="261" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>2025</v>
       </c>
@@ -30991,7 +30991,7 @@
         <v>1816</v>
       </c>
     </row>
-    <row r="277" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>2025</v>
       </c>
@@ -31267,7 +31267,7 @@
         <v>1859</v>
       </c>
     </row>
-    <row r="283" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>2025</v>
       </c>
@@ -31531,7 +31531,7 @@
         <v>1901</v>
       </c>
     </row>
-    <row r="289" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>2025</v>
       </c>
@@ -31945,7 +31945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>2025</v>
       </c>
@@ -32141,7 +32141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>2025</v>
       </c>
@@ -32572,7 +32572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>2025</v>
       </c>
@@ -32669,7 +32669,7 @@
         <v>2064</v>
       </c>
     </row>
-    <row r="315" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>2025</v>
       </c>
@@ -32810,7 +32810,7 @@
         <v>2085</v>
       </c>
     </row>
-    <row r="318" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>2025</v>
       </c>
@@ -33083,7 +33083,7 @@
         <v>2126</v>
       </c>
     </row>
-    <row r="324" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A324">
         <v>2025</v>
       </c>
@@ -33306,7 +33306,7 @@
         <v>2161</v>
       </c>
     </row>
-    <row r="329" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A329">
         <v>2025</v>
       </c>
@@ -33579,7 +33579,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="335" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335">
         <v>2025</v>
       </c>
@@ -33711,7 +33711,7 @@
         <v>2225</v>
       </c>
     </row>
-    <row r="338" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A338">
         <v>2025</v>
       </c>
@@ -34198,7 +34198,7 @@
         <v>2298</v>
       </c>
     </row>
-    <row r="349" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A349">
         <v>2025</v>
       </c>
@@ -34280,7 +34280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="351" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351">
         <v>2025</v>
       </c>
@@ -34424,7 +34424,7 @@
         <v>2328</v>
       </c>
     </row>
-    <row r="354" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A354">
         <v>2025</v>
       </c>
@@ -34585,7 +34585,7 @@
         <v>2354</v>
       </c>
     </row>
-    <row r="358" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358">
         <v>2025</v>
       </c>
@@ -35072,7 +35072,7 @@
         <v>2428</v>
       </c>
     </row>
-    <row r="369" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A369">
         <v>2025</v>
       </c>
@@ -35527,7 +35527,7 @@
         <v>2502</v>
       </c>
     </row>
-    <row r="379" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A379">
         <v>2025</v>
       </c>
@@ -35779,7 +35779,7 @@
         <v>2540</v>
       </c>
     </row>
-    <row r="385" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A385">
         <v>2025</v>
       </c>
@@ -35858,7 +35858,7 @@
         <v>2553</v>
       </c>
     </row>
-    <row r="387" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A387">
         <v>2025</v>
       </c>
@@ -35946,7 +35946,7 @@
         <v>2567</v>
       </c>
     </row>
-    <row r="389" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A389">
         <v>2025</v>
       </c>
@@ -35996,7 +35996,7 @@
         <v>2575</v>
       </c>
     </row>
-    <row r="390" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A390">
         <v>2025</v>
       </c>
@@ -36037,7 +36037,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="391" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A391">
         <v>2025</v>
       </c>
@@ -36210,7 +36210,7 @@
         <v>2610</v>
       </c>
     </row>
-    <row r="395" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A395">
         <v>2025</v>
       </c>
@@ -36307,7 +36307,7 @@
         <v>2623</v>
       </c>
     </row>
-    <row r="397" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A397">
         <v>2025</v>
       </c>
@@ -36357,7 +36357,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="398" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A398">
         <v>2025</v>
       </c>
@@ -36448,7 +36448,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="400" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A400">
         <v>2025</v>
       </c>
@@ -36498,7 +36498,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="401" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A401">
         <v>2025</v>
       </c>
@@ -36636,7 +36636,7 @@
         <v>2675</v>
       </c>
     </row>
-    <row r="404" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A404">
         <v>2025</v>
       </c>
@@ -36777,7 +36777,7 @@
         <v>2697</v>
       </c>
     </row>
-    <row r="407" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A407">
         <v>2025</v>
       </c>
@@ -37061,7 +37061,7 @@
         <v>2732</v>
       </c>
     </row>
-    <row r="414" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A414">
         <v>2025</v>
       </c>
@@ -37366,7 +37366,7 @@
         <v>2772</v>
       </c>
     </row>
-    <row r="421" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A421">
         <v>2025</v>
       </c>
@@ -38097,7 +38097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="437" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A437">
         <v>2025</v>
       </c>
@@ -38493,7 +38493,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="446" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A446">
         <v>2025</v>
       </c>
@@ -38543,7 +38543,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="447" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A447">
         <v>2025</v>
       </c>
@@ -38596,7 +38596,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="448" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A448">
         <v>2025</v>
       </c>
@@ -38687,9 +38687,15 @@
   </sheetData>
   <autoFilter ref="AF1:AF449" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="0">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
+      <filters>
+        <filter val="Ambiguous equity term (e.g. grassroots) with no paired ethnic signal"/>
+        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (African Origins) - verify manually"/>
+        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (African Origins, Caribbean Origins) - verify manually"/>
+        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (African Origins, European Origins) - verify manually"/>
+        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (Asian Origins) - verify manually"/>
+        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (Caribbean Origins) - verify manually"/>
+        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (European Origins) - verify manually"/>
+      </filters>
     </filterColumn>
   </autoFilter>
   <dataValidations count="4">

</xml_diff>

<commit_message>
Interim building upon classification flag expansion
</commit_message>
<xml_diff>
--- a/FR testing.xlsx
+++ b/FR testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myecf-my.sharepoint.com/personal/oadode_ecf_ca/Documents/Desktop/Discretionary FR Scripting/ECF-Discretionary-FR-Scripting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="11_1AE67D4D96B88102FD7E0298CDC6DCCA3A23EDAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BA90E4F-7B1B-4E75-8B7B-EA1BFA7F02FF}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_1AE67D4D96B88102FD7E0298CDC6DCCA3A23EDAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5C237F4-B3AC-4C37-8F24-DADA32ABF2B0}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19485,7 +19485,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2025</v>
       </c>
@@ -19535,7 +19535,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2025</v>
       </c>
@@ -19629,7 +19629,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="14" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2025</v>
       </c>
@@ -19676,7 +19676,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2025</v>
       </c>
@@ -19972,7 +19972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2025</v>
       </c>
@@ -21201,7 +21201,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="50" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>2025</v>
       </c>
@@ -22585,7 +22585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>2025</v>
       </c>
@@ -24264,7 +24264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>2025</v>
       </c>
@@ -24396,7 +24396,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="122" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>2025</v>
       </c>
@@ -24449,7 +24449,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="123" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>2025</v>
       </c>
@@ -24657,7 +24657,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="128" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>2025</v>
       </c>
@@ -24923,7 +24923,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="135" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>2025</v>
       </c>
@@ -24999,7 +24999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>2025</v>
       </c>
@@ -26021,7 +26021,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="162" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>2025</v>
       </c>
@@ -26121,7 +26121,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="164" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>2025</v>
       </c>
@@ -26707,7 +26707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>2025</v>
       </c>
@@ -27282,7 +27282,7 @@
         <v>1274</v>
       </c>
     </row>
-    <row r="191" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>2025</v>
       </c>
@@ -27951,7 +27951,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="206" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>2025</v>
       </c>
@@ -28432,7 +28432,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="217" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>2025</v>
       </c>
@@ -28661,7 +28661,7 @@
         <v>1473</v>
       </c>
     </row>
-    <row r="222" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>2025</v>
       </c>
@@ -28702,7 +28702,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="223" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>2025</v>
       </c>
@@ -28743,7 +28743,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="224" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>2025</v>
       </c>
@@ -29010,7 +29010,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="230" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>2025</v>
       </c>
@@ -29110,7 +29110,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="232" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>2025</v>
       </c>
@@ -29160,7 +29160,7 @@
         <v>884</v>
       </c>
     </row>
-    <row r="233" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>2025</v>
       </c>
@@ -29515,7 +29515,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="241" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>2025</v>
       </c>
@@ -30196,7 +30196,7 @@
         <v>1693</v>
       </c>
     </row>
-    <row r="259" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>2025</v>
       </c>
@@ -30290,7 +30290,7 @@
         <v>1705</v>
       </c>
     </row>
-    <row r="261" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>2025</v>
       </c>
@@ -31581,7 +31581,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="290" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>2025</v>
       </c>
@@ -31766,7 +31766,7 @@
         <v>1933</v>
       </c>
     </row>
-    <row r="294" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>2025</v>
       </c>
@@ -32241,7 +32241,7 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="305" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>2025</v>
       </c>
@@ -32810,7 +32810,7 @@
         <v>2085</v>
       </c>
     </row>
-    <row r="318" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>2025</v>
       </c>
@@ -34280,7 +34280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="351" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A351">
         <v>2025</v>
       </c>
@@ -34333,7 +34333,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="352" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A352">
         <v>2025</v>
       </c>
@@ -35527,7 +35527,7 @@
         <v>2502</v>
       </c>
     </row>
-    <row r="379" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A379">
         <v>2025</v>
       </c>
@@ -35858,7 +35858,7 @@
         <v>2553</v>
       </c>
     </row>
-    <row r="387" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A387">
         <v>2025</v>
       </c>
@@ -36970,7 +36970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="412" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A412">
         <v>2025</v>
       </c>
@@ -37636,7 +37636,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="427" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A427">
         <v>2025</v>
       </c>
@@ -37771,7 +37771,7 @@
         <v>2829</v>
       </c>
     </row>
-    <row r="430" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A430">
         <v>2025</v>
       </c>
@@ -38443,7 +38443,7 @@
         <v>2932</v>
       </c>
     </row>
-    <row r="445" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
       <c r="A445">
         <v>2025</v>
       </c>
@@ -38596,7 +38596,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="448" spans="1:32" hidden="1" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A448">
         <v>2025</v>
       </c>
@@ -38688,13 +38688,7 @@
   <autoFilter ref="AF1:AF449" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Ambiguous equity term (e.g. grassroots) with no paired ethnic signal"/>
-        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (African Origins) - verify manually"/>
-        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (African Origins, Caribbean Origins) - verify manually"/>
-        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (African Origins, European Origins) - verify manually"/>
-        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (Asian Origins) - verify manually"/>
-        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (Caribbean Origins) - verify manually"/>
-        <filter val="Ambiguous: BIPOC mentioned alongside specific group(s) (European Origins) - verify manually"/>
+        <filter val="BIPOC target detected"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>